<commit_message>
top 19 cutoff update
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U52"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,11 @@
           <t>Rank 18</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Rank 19</t>
+        </is>
+      </c>
     </row>
     <row r="2"/>
     <row r="3">
@@ -555,10 +560,10 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0.638</v>
+        <v>0.605</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0.362</v>
+        <v>0.395</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
@@ -576,6 +581,7 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -590,16 +596,16 @@
         <v>2</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.362</v>
+        <v>0.395</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.58</v>
+        <v>0.544</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>0.054</v>
+        <v>0.058</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -615,11 +621,12 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Я ненавижу покер v.2</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -630,19 +637,23 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" s="1" t="n">
-        <v>0.056</v>
+        <v>0.001</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>0.855</v>
+        <v>0.05</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.506</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+        <v>0.276</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>0.027</v>
+      </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
@@ -654,11 +665,12 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>Антуан Гризманн</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -668,27 +680,33 @@
         <v>4</v>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="F6" s="1" t="n">
-        <v>0.049</v>
+        <v>0.03</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>0.494</v>
+        <v>0.311</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>0.296</v>
+        <v>0.28</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>0.144</v>
+        <v>0.074</v>
       </c>
       <c r="J6" s="1" t="n">
-        <v>0.015</v>
+        <v>0.15</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+        <v>0.114</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="M6" s="1" t="n">
+        <v>0.006</v>
+      </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -697,11 +715,12 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Антуан Гризманн</t>
+          <t>E_ishutkin</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -711,36 +730,30 @@
         <v>5</v>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>0.042</v>
-      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" s="1" t="n">
-        <v>0.315</v>
+        <v>0.103</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>0.246</v>
+        <v>0.364</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>0.068</v>
+        <v>0.387</v>
       </c>
       <c r="J7" s="1" t="n">
-        <v>0.146</v>
+        <v>0.083</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>0.128</v>
+        <v>0.045</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>0.051</v>
+        <v>0.017</v>
       </c>
       <c r="M7" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="N7" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
@@ -748,11 +761,12 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>E_ishutkin</t>
+          <t>clayzid</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
@@ -765,39 +779,52 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" s="1" t="n">
-        <v>0.094</v>
+        <v>0.003</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>0.37</v>
+        <v>0.057</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>0.4</v>
+        <v>0.255</v>
       </c>
       <c r="J8" s="1" t="n">
-        <v>0.1</v>
+        <v>0.306</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>0.028</v>
+        <v>0.039</v>
       </c>
       <c r="L8" s="1" t="n">
-        <v>0.006</v>
+        <v>0.029</v>
       </c>
       <c r="M8" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+        <v>0.057</v>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="O8" s="1" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="P8" s="1" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="Q8" s="1" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R8" s="1" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="S8" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>clayzid</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -809,50 +836,57 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" s="1" t="n">
-        <v>0.008</v>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" s="1" t="n">
-        <v>0.061</v>
+        <v>0.012</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>0.256</v>
+        <v>0.049</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>0.298</v>
+        <v>0.138</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>0.049</v>
+        <v>0.204</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>0.024</v>
+        <v>0.128</v>
       </c>
       <c r="M9" s="1" t="n">
-        <v>0.056</v>
+        <v>0.066</v>
       </c>
       <c r="N9" s="1" t="n">
-        <v>0.081</v>
+        <v>0.03</v>
       </c>
       <c r="O9" s="1" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="P9" s="1" t="n">
-        <v>0.053</v>
+        <v>0.006</v>
       </c>
       <c r="Q9" s="1" t="n">
-        <v>0.022</v>
+        <v>0.005</v>
       </c>
       <c r="R9" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+        <v>0.048</v>
+      </c>
+      <c r="S9" s="1" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="T9" s="1" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="U9" s="1" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="V9" s="1" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>В азарт не входим</t>
+          <t>Котяра</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -865,47 +899,52 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="1" t="n">
-        <v>0.014</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>0.056</v>
+        <v>0.003</v>
       </c>
       <c r="J10" s="1" t="n">
-        <v>0.137</v>
+        <v>0.024</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>0.21</v>
+        <v>0.076</v>
       </c>
       <c r="L10" s="1" t="n">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="M10" s="1" t="n">
-        <v>0.149</v>
+        <v>0.159</v>
       </c>
       <c r="N10" s="1" t="n">
-        <v>0.136</v>
+        <v>0.159</v>
       </c>
       <c r="O10" s="1" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.119</v>
       </c>
       <c r="P10" s="1" t="n">
-        <v>0.034</v>
+        <v>0.111</v>
       </c>
       <c r="Q10" s="1" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="R10" s="1" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="S10" s="1" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="T10" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="U10" s="1" t="n">
         <v>0.004</v>
       </c>
-      <c r="R10" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Котяра</t>
+          <t>Кинзу</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
@@ -919,48 +958,51 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" s="1" t="n">
+        <v>0.004</v>
+      </c>
       <c r="J11" s="1" t="n">
-        <v>0.023</v>
+        <v>0.021</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>0.092</v>
+        <v>0.09</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>0.159</v>
+        <v>0.112</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>0.174</v>
+        <v>0.139</v>
       </c>
       <c r="N11" s="1" t="n">
-        <v>0.153</v>
+        <v>0.114</v>
       </c>
       <c r="O11" s="1" t="n">
-        <v>0.1</v>
+        <v>0.106</v>
       </c>
       <c r="P11" s="1" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.098</v>
       </c>
       <c r="Q11" s="1" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="R11" s="1" t="n">
         <v>0.091</v>
       </c>
-      <c r="R11" s="1" t="n">
-        <v>0.054</v>
-      </c>
       <c r="S11" s="1" t="n">
-        <v>0.045</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T11" s="1" t="n">
-        <v>0.02</v>
+        <v>0.037</v>
       </c>
       <c r="U11" s="1" t="n">
-        <v>0.004</v>
-      </c>
+        <v>0.005</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Кинзу</t>
+          <t>дисциплина</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -975,112 +1017,96 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>0.003</v>
+        <v>0.007</v>
       </c>
       <c r="J12" s="1" t="n">
-        <v>0.021</v>
+        <v>0.042</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.063</v>
       </c>
       <c r="L12" s="1" t="n">
-        <v>0.129</v>
+        <v>0.124</v>
       </c>
       <c r="M12" s="1" t="n">
-        <v>0.142</v>
+        <v>0.109</v>
       </c>
       <c r="N12" s="1" t="n">
-        <v>0.12</v>
+        <v>0.113</v>
       </c>
       <c r="O12" s="1" t="n">
-        <v>0.114</v>
+        <v>0.092</v>
       </c>
       <c r="P12" s="1" t="n">
-        <v>0.103</v>
+        <v>0.096</v>
       </c>
       <c r="Q12" s="1" t="n">
-        <v>0.103</v>
+        <v>0.113</v>
       </c>
       <c r="R12" s="1" t="n">
-        <v>0.096</v>
+        <v>0.112</v>
       </c>
       <c r="S12" s="1" t="n">
-        <v>0.061</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="T12" s="1" t="n">
-        <v>0.032</v>
+        <v>0.04</v>
       </c>
       <c r="U12" s="1" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
+      </c>
+      <c r="V12" s="1" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>дисциплина</t>
+          <t>Я ненавижу покер v.2</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="C13" t="n">
         <v>11</v>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="E13" s="1" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>0.074</v>
+      </c>
       <c r="H13" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="I13" s="1" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="J13" s="1" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="K13" s="1" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="L13" s="1" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="M13" s="1" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="N13" s="1" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="O13" s="1" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="P13" s="1" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="Q13" s="1" t="n">
-        <v>0.117</v>
-      </c>
-      <c r="R13" s="1" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="S13" s="1" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="T13" s="1" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="U13" s="1" t="n">
-        <v>0.007</v>
-      </c>
+        <v>0.005</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ksuhony</t>
+          <t>В азарт не входим</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="C14" t="n">
         <v>12</v>
@@ -1089,51 +1115,50 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="H14" s="1" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="I14" s="1" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>0.15</v>
+      </c>
       <c r="K14" s="1" t="n">
-        <v>0.005</v>
+        <v>0.202</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>0.01</v>
+        <v>0.182</v>
       </c>
       <c r="M14" s="1" t="n">
-        <v>0.025</v>
+        <v>0.164</v>
       </c>
       <c r="N14" s="1" t="n">
-        <v>0.052</v>
+        <v>0.121</v>
       </c>
       <c r="O14" s="1" t="n">
-        <v>0.094</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="P14" s="1" t="n">
-        <v>0.172</v>
+        <v>0.034</v>
       </c>
       <c r="Q14" s="1" t="n">
-        <v>0.194</v>
-      </c>
-      <c r="R14" s="1" t="n">
-        <v>0.168</v>
-      </c>
-      <c r="S14" s="1" t="n">
-        <v>0.163</v>
-      </c>
-      <c r="T14" s="1" t="n">
-        <v>0.092</v>
-      </c>
-      <c r="U14" s="1" t="n">
-        <v>0.025</v>
-      </c>
+        <v>0.007</v>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>ksuhony</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.994</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="C15" t="n">
         <v>13</v>
@@ -1142,48 +1167,43 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="1" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="I15" s="1" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="J15" s="1" t="n">
-        <v>0.146</v>
-      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" s="1" t="n">
-        <v>0.193</v>
+        <v>0.002</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>0.119</v>
+        <v>0.013</v>
       </c>
       <c r="M15" s="1" t="n">
-        <v>0.06</v>
+        <v>0.026</v>
       </c>
       <c r="N15" s="1" t="n">
-        <v>0.014</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="O15" s="1" t="n">
-        <v>0.011</v>
+        <v>0.095</v>
       </c>
       <c r="P15" s="1" t="n">
-        <v>0.008</v>
+        <v>0.144</v>
       </c>
       <c r="Q15" s="1" t="n">
-        <v>0.017</v>
+        <v>0.18</v>
       </c>
       <c r="R15" s="1" t="n">
-        <v>0.054</v>
+        <v>0.178</v>
       </c>
       <c r="S15" s="1" t="n">
-        <v>0.125</v>
+        <v>0.17</v>
       </c>
       <c r="T15" s="1" t="n">
-        <v>0.127</v>
+        <v>0.097</v>
       </c>
       <c r="U15" s="1" t="n">
-        <v>0.061</v>
-      </c>
+        <v>0.024</v>
+      </c>
+      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1192,7 +1212,7 @@
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.98</v>
+        <v>0.9989999999999999</v>
       </c>
       <c r="C16" t="n">
         <v>14</v>
@@ -1204,46 +1224,51 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="L16" s="1" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="M16" s="1" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
       <c r="N16" s="1" t="n">
-        <v>0.023</v>
+        <v>0.017</v>
       </c>
       <c r="O16" s="1" t="n">
-        <v>0.042</v>
+        <v>0.036</v>
       </c>
       <c r="P16" s="1" t="n">
-        <v>0.079</v>
+        <v>0.063</v>
       </c>
       <c r="Q16" s="1" t="n">
-        <v>0.091</v>
+        <v>0.114</v>
       </c>
       <c r="R16" s="1" t="n">
-        <v>0.151</v>
+        <v>0.146</v>
       </c>
       <c r="S16" s="1" t="n">
-        <v>0.209</v>
+        <v>0.219</v>
       </c>
       <c r="T16" s="1" t="n">
-        <v>0.244</v>
+        <v>0.236</v>
       </c>
       <c r="U16" s="1" t="n">
-        <v>0.133</v>
+        <v>0.14</v>
+      </c>
+      <c r="V16" s="1" t="n">
+        <v>0.019</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Niko</t>
+          <t>yakushevass</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.9610000000000001</v>
+        <v>0.996</v>
       </c>
       <c r="C17" t="n">
         <v>15</v>
@@ -1255,50 +1280,53 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" s="1" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="K17" s="1" t="n">
-        <v>0.017</v>
+        <v>0.036</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>0.037</v>
+        <v>0.076</v>
       </c>
       <c r="M17" s="1" t="n">
-        <v>0.058</v>
+        <v>0.093</v>
       </c>
       <c r="N17" s="1" t="n">
-        <v>0.093</v>
+        <v>0.113</v>
       </c>
       <c r="O17" s="1" t="n">
-        <v>0.142</v>
+        <v>0.137</v>
       </c>
       <c r="P17" s="1" t="n">
-        <v>0.136</v>
+        <v>0.129</v>
       </c>
       <c r="Q17" s="1" t="n">
-        <v>0.144</v>
+        <v>0.065</v>
       </c>
       <c r="R17" s="1" t="n">
-        <v>0.135</v>
+        <v>0.05</v>
       </c>
       <c r="S17" s="1" t="n">
-        <v>0.078</v>
+        <v>0.057</v>
       </c>
       <c r="T17" s="1" t="n">
-        <v>0.052</v>
+        <v>0.089</v>
       </c>
       <c r="U17" s="1" t="n">
-        <v>0.063</v>
+        <v>0.117</v>
+      </c>
+      <c r="V17" s="1" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>yakushevass</t>
+          <t>Niko</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.9600000000000001</v>
+        <v>0.9950000000000001</v>
       </c>
       <c r="C18" t="n">
         <v>16</v>
@@ -1310,40 +1338,43 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" s="1" t="n">
-        <v>0.013</v>
+        <v>0.005</v>
       </c>
       <c r="K18" s="1" t="n">
-        <v>0.025</v>
+        <v>0.017</v>
       </c>
       <c r="L18" s="1" t="n">
-        <v>0.062</v>
+        <v>0.034</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="N18" s="1" t="n">
-        <v>0.122</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O18" s="1" t="n">
-        <v>0.151</v>
+        <v>0.133</v>
       </c>
       <c r="P18" s="1" t="n">
-        <v>0.124</v>
+        <v>0.15</v>
       </c>
       <c r="Q18" s="1" t="n">
-        <v>0.08</v>
+        <v>0.168</v>
       </c>
       <c r="R18" s="1" t="n">
-        <v>0.049</v>
+        <v>0.136</v>
       </c>
       <c r="S18" s="1" t="n">
-        <v>0.054</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="T18" s="1" t="n">
-        <v>0.092</v>
+        <v>0.061</v>
       </c>
       <c r="U18" s="1" t="n">
-        <v>0.101</v>
+        <v>0.061</v>
+      </c>
+      <c r="V18" s="1" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="19">
@@ -1353,7 +1384,7 @@
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.893</v>
+        <v>0.986</v>
       </c>
       <c r="C19" t="n">
         <v>17</v>
@@ -1362,143 +1393,150 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="K19" s="1" t="n">
-        <v>0.116</v>
+        <v>0.11</v>
       </c>
       <c r="L19" s="1" t="n">
         <v>0.118</v>
       </c>
       <c r="M19" s="1" t="n">
-        <v>0.109</v>
+        <v>0.12</v>
       </c>
       <c r="N19" s="1" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.095</v>
       </c>
       <c r="O19" s="1" t="n">
-        <v>0.054</v>
+        <v>0.078</v>
       </c>
       <c r="P19" s="1" t="n">
-        <v>0.054</v>
+        <v>0.043</v>
       </c>
       <c r="Q19" s="1" t="n">
-        <v>0.033</v>
+        <v>0.036</v>
       </c>
       <c r="R19" s="1" t="n">
         <v>0.022</v>
       </c>
       <c r="S19" s="1" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="T19" s="1" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="U19" s="1" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="V19" s="1" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ПокерНЕок</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>0.623</v>
+      </c>
+      <c r="C20" t="n">
+        <v>18</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" s="1" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="Q20" s="1" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="R20" s="1" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="S20" s="1" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="T20" s="1" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="U20" s="1" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="V20" s="1" t="n">
+        <v>0.277</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Добросердечный</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="Q21" s="3" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="S21" s="3" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="T21" s="3" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="U21" s="3" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="V21" s="3" t="n">
         <v>0.016</v>
-      </c>
-      <c r="T19" s="1" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="U19" s="1" t="n">
-        <v>0.126</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Добросердечный</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="3" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="M20" s="3" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="N20" s="3" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="O20" s="3" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="P20" s="3" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="Q20" s="3" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="R20" s="3" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="S20" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="T20" s="3" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="U20" s="3" t="n">
-        <v>0.034</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>ПокерНЕок</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>0.388</v>
-      </c>
-      <c r="C21" t="n">
-        <v>19</v>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="P21" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="Q21" s="1" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="R21" s="1" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="S21" s="1" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="T21" s="1" t="n">
-        <v>0.101</v>
-      </c>
-      <c r="U21" s="1" t="n">
-        <v>0.215</v>
       </c>
     </row>
     <row r="22">
@@ -1508,7 +1546,7 @@
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.167</v>
+        <v>0.31</v>
       </c>
       <c r="C22" t="n">
         <v>20</v>
@@ -1524,9 +1562,7 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" s="1" t="n">
         <v>0.001</v>
@@ -1535,13 +1571,16 @@
         <v>0.007</v>
       </c>
       <c r="S22" s="1" t="n">
-        <v>0.013</v>
+        <v>0.016</v>
       </c>
       <c r="T22" s="1" t="n">
         <v>0.041</v>
       </c>
       <c r="U22" s="1" t="n">
-        <v>0.104</v>
+        <v>0.099</v>
+      </c>
+      <c r="V22" s="1" t="n">
+        <v>0.146</v>
       </c>
     </row>
     <row r="23">
@@ -1551,7 +1590,7 @@
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.306</v>
       </c>
       <c r="C23" t="n">
         <v>21</v>
@@ -1571,12 +1610,17 @@
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="T23" s="1" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="U23" s="1" t="n">
-        <v>0.067</v>
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="V23" s="1" t="n">
+        <v>0.233</v>
       </c>
     </row>
     <row r="24">
@@ -1586,7 +1630,7 @@
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>0.053</v>
+        <v>0.217</v>
       </c>
       <c r="C24" t="n">
         <v>22</v>
@@ -1608,10 +1652,13 @@
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" s="1" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="U24" s="1" t="n">
-        <v>0.051</v>
+        <v>0.062</v>
+      </c>
+      <c r="V24" s="1" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="25">
@@ -1621,7 +1668,7 @@
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>0.004</v>
+        <v>0.017</v>
       </c>
       <c r="C25" t="n">
         <v>23</v>
@@ -1643,17 +1690,20 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" s="1" t="n">
-        <v>0.004</v>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" s="1" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sl1dbygad</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>Сокол</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>0.003</v>
+      </c>
       <c r="C26" t="n">
         <v>24</v>
       </c>
@@ -1674,15 +1724,22 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="V26" s="1" t="n">
+        <v>0.002</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Сокол</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>Пассажир</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="C27" t="n">
         <v>25</v>
       </c>
@@ -1703,15 +1760,20 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
+      <c r="U27" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="V27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Пассажир</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>sl1dbygad</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="C28" t="n">
         <v>26</v>
       </c>
@@ -1732,12 +1794,15 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="V28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>EliasPavlov</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1762,11 +1827,12 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>EliasPavlov</t>
+          <t>rusya6996</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1791,11 +1857,12 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Викусик</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1820,11 +1887,12 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Кальян</t>
+          <t>Плейбой в карты</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1849,11 +1917,12 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Плейбой в карты</t>
+          <t>Викусик</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1878,11 +1947,12 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Дядя Витя</t>
+          <t>Кальян</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1907,11 +1977,12 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1936,11 +2007,12 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>Дядя Витя</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1965,11 +2037,12 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1994,11 +2067,12 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>nesmotri_v_shelll1</t>
+          <t>maria_merlot</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -2023,11 +2097,12 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>finch79</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -2052,11 +2127,12 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>rusya6996</t>
+          <t>nesmotri_v_shelll1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -2081,11 +2157,12 @@
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>maria_merlot</t>
+          <t>Chesters</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -2110,6 +2187,7 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2139,11 +2217,12 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Тихоня</t>
+          <t>cheremsha</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -2168,11 +2247,12 @@
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Chinaski</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2197,11 +2277,12 @@
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Chinaski</t>
+          <t>@TryFraiz</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -2226,11 +2307,12 @@
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Chesters</t>
+          <t>finch79</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -2255,11 +2337,12 @@
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cheremsha</t>
+          <t>Тихоня</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -2284,11 +2367,12 @@
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>@TryFraiz</t>
+          <t>yankkk</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -2313,11 +2397,12 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>yankkk</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -2342,6 +2427,7 @@
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2371,11 +2457,12 @@
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>Кесадилия</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2400,11 +2487,12 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Кесадилия</t>
+          <t>Никитос</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2429,6 +2517,7 @@
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B52">
@@ -2443,7 +2532,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:U52">
+  <conditionalFormatting sqref="D2:V52">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2457,7 +2546,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:C52">
     <cfRule type="cellIs" priority="3" operator="lessThanOrEqual" dxfId="0">
-      <formula>18</formula>
+      <formula>19</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
end of april season
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V52"/>
+  <dimension ref="A1:U52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -540,17 +540,12 @@
           <t>Rank 18</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Rank 19</t>
-        </is>
-      </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Roman_Furtatov</t>
+          <t>ПокерНЕок</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -559,12 +554,8 @@
       <c r="C3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="1" t="n">
-        <v>0.605</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>0.395</v>
-      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -580,13 +571,14 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="U3" s="1" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Руслан</t>
+          <t>Roman_Furtatov</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -596,17 +588,11 @@
         <v>2</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.395</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>0.003</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -621,12 +607,11 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>Руслан</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -637,23 +622,13 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>0.506</v>
-      </c>
-      <c r="H5" s="1" t="n">
-        <v>0.276</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>0.027</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
@@ -665,12 +640,11 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Антуан Гризманн</t>
+          <t>Я ненавижу покер v.2</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -680,33 +654,17 @@
         <v>4</v>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" s="1" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>0.311</v>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="L6" s="1" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0.006</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -715,12 +673,11 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>E_ishutkin</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -733,26 +690,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" s="1" t="n">
-        <v>0.103</v>
-      </c>
-      <c r="H7" s="1" t="n">
-        <v>0.364</v>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>0.387</v>
-      </c>
-      <c r="J7" s="1" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="K7" s="1" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="L7" s="1" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="M7" s="1" t="n">
-        <v>0.001</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -761,12 +706,11 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>clayzid</t>
+          <t>E_ishutkin</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
@@ -778,53 +722,28 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" s="1" t="n">
-        <v>0.003</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" s="1" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>0.255</v>
-      </c>
-      <c r="J8" s="1" t="n">
-        <v>0.306</v>
-      </c>
-      <c r="K8" s="1" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="L8" s="1" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="M8" s="1" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="N8" s="1" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="O8" s="1" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="P8" s="1" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="Q8" s="1" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="R8" s="1" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="S8" s="1" t="n">
-        <v>0.001</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>Антуан Гризманн</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -837,56 +756,27 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="n">
-        <v>0.012</v>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="J9" s="1" t="n">
-        <v>0.138</v>
-      </c>
-      <c r="K9" s="1" t="n">
-        <v>0.204</v>
-      </c>
-      <c r="L9" s="1" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="M9" s="1" t="n">
-        <v>0.066</v>
-      </c>
-      <c r="N9" s="1" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="O9" s="1" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="P9" s="1" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="Q9" s="1" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="R9" s="1" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="S9" s="1" t="n">
-        <v>0.103</v>
-      </c>
-      <c r="T9" s="1" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="U9" s="1" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="V9" s="1" t="n">
-        <v>0.003</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Котяра</t>
+          <t>В азарт не входим</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -900,46 +790,21 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" s="1" t="n">
-        <v>0.003</v>
-      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" s="1" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="L10" s="1" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="M10" s="1" t="n">
-        <v>0.159</v>
-      </c>
-      <c r="N10" s="1" t="n">
-        <v>0.159</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>0.119</v>
-      </c>
-      <c r="P10" s="1" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="Q10" s="1" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="R10" s="1" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="S10" s="1" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="T10" s="1" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="U10" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="V10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -958,51 +823,26 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="J11" s="1" t="n">
-        <v>0.021</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" s="1" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="L11" s="1" t="n">
-        <v>0.112</v>
-      </c>
-      <c r="M11" s="1" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="N11" s="1" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="O11" s="1" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="P11" s="1" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="Q11" s="1" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="R11" s="1" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="S11" s="1" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="T11" s="1" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="U11" s="1" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="V11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>дисциплина</t>
+          <t>clayzid</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -1016,79 +856,46 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" s="1" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>0.063</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" s="1" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="M12" s="1" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="N12" s="1" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="O12" s="1" t="n">
-        <v>0.092</v>
-      </c>
-      <c r="P12" s="1" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="Q12" s="1" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="R12" s="1" t="n">
-        <v>0.112</v>
-      </c>
-      <c r="S12" s="1" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="T12" s="1" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="U12" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="V12" s="1" t="n">
-        <v>0.001</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Я ненавижу покер v.2</t>
+          <t>Бэндер</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
         <v>11</v>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" s="1" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="F13" s="1" t="n">
-        <v>0.862</v>
-      </c>
-      <c r="G13" s="1" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="H13" s="1" t="n">
-        <v>0.005</v>
-      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -1097,16 +904,15 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>В азарт не входим</t>
+          <t>дисциплина</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="C14" t="n">
         <v>12</v>
@@ -1115,41 +921,22 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="I14" s="1" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K14" s="1" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="L14" s="1" t="n">
-        <v>0.182</v>
-      </c>
-      <c r="M14" s="1" t="n">
-        <v>0.164</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" s="1" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="O14" s="1" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="P14" s="1" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="Q14" s="1" t="n">
-        <v>0.007</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1158,7 +945,7 @@
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
         <v>13</v>
@@ -1170,49 +957,28 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="L15" s="1" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="M15" s="1" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="N15" s="1" t="n">
-        <v>0.07099999999999999</v>
-      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" s="1" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="P15" s="1" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="Q15" s="1" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="R15" s="1" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="S15" s="1" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="T15" s="1" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="U15" s="1" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="V15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kanti</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.9989999999999999</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
         <v>14</v>
@@ -1224,51 +990,28 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="L16" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="M16" s="1" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="O16" s="1" t="n">
-        <v>0.036</v>
-      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
       <c r="P16" s="1" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="Q16" s="1" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="R16" s="1" t="n">
-        <v>0.146</v>
-      </c>
-      <c r="S16" s="1" t="n">
-        <v>0.219</v>
-      </c>
-      <c r="T16" s="1" t="n">
-        <v>0.236</v>
-      </c>
-      <c r="U16" s="1" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="V16" s="1" t="n">
-        <v>0.019</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>yakushevass</t>
+          <t>Kanti</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
         <v>15</v>
@@ -1279,54 +1022,29 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="K17" s="1" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="L17" s="1" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="M17" s="1" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="N17" s="1" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="O17" s="1" t="n">
-        <v>0.137</v>
-      </c>
-      <c r="P17" s="1" t="n">
-        <v>0.129</v>
-      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
       <c r="Q17" s="1" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="R17" s="1" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="S17" s="1" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="T17" s="1" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="U17" s="1" t="n">
-        <v>0.117</v>
-      </c>
-      <c r="V17" s="1" t="n">
-        <v>0.03</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Niko</t>
+          <t>yakushevass</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.9950000000000001</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
         <v>16</v>
@@ -1337,54 +1055,29 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="1" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="K18" s="1" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="M18" s="1" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="N18" s="1" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="O18" s="1" t="n">
-        <v>0.133</v>
-      </c>
-      <c r="P18" s="1" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Q18" s="1" t="n">
-        <v>0.168</v>
-      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" s="1" t="n">
-        <v>0.136</v>
-      </c>
-      <c r="S18" s="1" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="T18" s="1" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="U18" s="1" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="V18" s="1" t="n">
-        <v>0.026</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Бэндер</t>
+          <t>Котяра</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.986</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
         <v>17</v>
@@ -1394,150 +1087,83 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" s="1" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="J19" s="1" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="K19" s="1" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="L19" s="1" t="n">
-        <v>0.118</v>
-      </c>
-      <c r="M19" s="1" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="N19" s="1" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="O19" s="1" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="P19" s="1" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="Q19" s="1" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="R19" s="1" t="n">
-        <v>0.022</v>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
       <c r="S19" s="1" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="T19" s="1" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="U19" s="1" t="n">
-        <v>0.134</v>
-      </c>
-      <c r="V19" s="1" t="n">
-        <v>0.08</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ПокерНЕок</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>0.623</v>
-      </c>
-      <c r="C20" t="n">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Niko</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" s="1" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="Q20" s="1" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="R20" s="1" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="S20" s="1" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="T20" s="1" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="U20" s="1" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="V20" s="1" t="n">
-        <v>0.277</v>
-      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Добросердечный</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
-        <v>0.546</v>
-      </c>
-      <c r="C21" s="2" t="n">
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="n">
         <v>19</v>
       </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="L21" s="3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M21" s="3" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="N21" s="3" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="O21" s="3" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="P21" s="3" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="R21" s="3" t="n">
-        <v>0.118</v>
-      </c>
-      <c r="S21" s="3" t="n">
-        <v>0.097</v>
-      </c>
-      <c r="T21" s="3" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="U21" s="3" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="V21" s="3" t="n">
-        <v>0.016</v>
-      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1545,9 +1171,7 @@
           <t>Mihmbox</t>
         </is>
       </c>
-      <c r="B22" s="1" t="n">
-        <v>0.31</v>
-      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>20</v>
       </c>
@@ -1564,34 +1188,19 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="R22" s="1" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="S22" s="1" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="T22" s="1" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="U22" s="1" t="n">
-        <v>0.099</v>
-      </c>
-      <c r="V22" s="1" t="n">
-        <v>0.146</v>
-      </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Obscur</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>0.306</v>
-      </c>
+          <t>Vitos2049</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>21</v>
       </c>
@@ -1610,28 +1219,17 @@
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="T23" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U23" s="1" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="V23" s="1" t="n">
-        <v>0.233</v>
-      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Vitos2049</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="n">
-        <v>0.217</v>
-      </c>
+          <t>Obscur</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>22</v>
       </c>
@@ -1651,15 +1249,8 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
-      <c r="T24" s="1" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="U24" s="1" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="V24" s="1" t="n">
-        <v>0.15</v>
-      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1667,9 +1258,7 @@
           <t>Amaney</t>
         </is>
       </c>
-      <c r="B25" s="1" t="n">
-        <v>0.017</v>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>23</v>
       </c>
@@ -1691,19 +1280,14 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" s="1" t="n">
-        <v>0.017</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Сокол</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="n">
-        <v>0.003</v>
-      </c>
+          <t>sl1dbygad</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>24</v>
       </c>
@@ -1724,22 +1308,15 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
-      <c r="U26" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="V26" s="1" t="n">
-        <v>0.002</v>
-      </c>
+      <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Пассажир</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="n">
-        <v>0.001</v>
-      </c>
+          <t>Викусик</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>25</v>
       </c>
@@ -1760,20 +1337,15 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sl1dbygad</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="n">
-        <v>0.001</v>
-      </c>
+          <t>Сокол</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>26</v>
       </c>
@@ -1794,15 +1366,12 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EliasPavlov</t>
+          <t>Плейбой в карты</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1827,12 +1396,11 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>rusya6996</t>
+          <t>Пассажир</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1857,12 +1425,11 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>Кальян</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1887,12 +1454,11 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Плейбой в карты</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1917,12 +1483,11 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Викусик</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1947,12 +1512,11 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Кальян</t>
+          <t>EliasPavlov</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1977,12 +1541,11 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>Дядя Витя</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -2007,12 +1570,11 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Дядя Витя</t>
+          <t>TryFraiz</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -2037,12 +1599,11 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -2067,12 +1628,11 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>maria_merlot</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -2097,12 +1657,11 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>nesmotri_v_shelll1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -2127,12 +1686,11 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>nesmotri_v_shelll1</t>
+          <t>rusya6996</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -2157,12 +1715,11 @@
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chesters</t>
+          <t>Bushido</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -2187,12 +1744,11 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Bushido</t>
+          <t>Сан Саныч</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -2217,12 +1773,11 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cheremsha</t>
+          <t>Никитос</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -2247,12 +1802,11 @@
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Chinaski</t>
+          <t>ЛЕНИН</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2277,12 +1831,11 @@
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>@TryFraiz</t>
+          <t>cheremsha</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -2307,12 +1860,11 @@
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>finch79</t>
+          <t>Chesters</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -2337,12 +1889,11 @@
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Тихоня</t>
+          <t>Комарик</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -2367,12 +1918,11 @@
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>yankkk</t>
+          <t>Chinaski</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -2397,12 +1947,11 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>finch79</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -2427,12 +1976,11 @@
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>АРАМАИСКА</t>
+          <t>Тихоня</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2457,12 +2005,11 @@
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Кесадилия</t>
+          <t>yankkk</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2487,12 +2034,11 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Никитос</t>
+          <t>maria_merlot</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2517,7 +2063,6 @@
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B52">
@@ -2532,7 +2077,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:V52">
+  <conditionalFormatting sqref="D2:U52">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2546,7 +2091,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:C52">
     <cfRule type="cellIs" priority="3" operator="lessThanOrEqual" dxfId="0">
-      <formula>19</formula>
+      <formula>18</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
FIXED START OF MAY WITH MULTIPLIERS
</commit_message>
<xml_diff>
--- a/data/playoff_odds.xlsx
+++ b/data/playoff_odds.xlsx
@@ -545,41 +545,41 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Noize MC</t>
+          <t>Гризли</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0.515</v>
+        <v>0.387</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0.287</v>
+        <v>0.343</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>0.164</v>
+        <v>0.222</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>0.019</v>
+        <v>0.03</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="J3" s="1" t="n">
         <v>0.002</v>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
@@ -592,32 +592,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Гризли</t>
+          <t>Драйв</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="C4" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.372</v>
+        <v>0.11</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.394</v>
+        <v>0.333</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>0.186</v>
+        <v>0.455</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>0.033</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>0.01</v>
+        <v>0.022</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>0.004</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="J4" s="1" t="n">
         <v>0.001</v>
@@ -637,43 +637,51 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Драйв</t>
+          <t>long_2203</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="C5" t="n">
         <v>3</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>0.112</v>
+        <v>0.001</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.3</v>
+        <v>0.013</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>0.467</v>
+        <v>0.134</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.507</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>0.028</v>
+        <v>0.201</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>0.016</v>
+        <v>0.108</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>0.004</v>
+        <v>0.024</v>
       </c>
       <c r="K5" s="1" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="L5" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" s="1" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="N5" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="O5" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
@@ -684,47 +692,41 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>long_2203</t>
+          <t>Noize MC</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>1</v>
+        <v>0.298</v>
       </c>
       <c r="C6" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="1" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="E6" s="1" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>0.142</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>0.511</v>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>0.018</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="L6" s="1" t="n">
-        <v>0.005</v>
-      </c>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
@@ -739,49 +741,45 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>1</v>
+        <v>0.297702</v>
       </c>
       <c r="C7" t="n">
         <v>5</v>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" s="1" t="n">
-        <v>0.002</v>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" s="1" t="n">
-        <v>0.031</v>
+        <v>0.026</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>0.217</v>
+        <v>0.216</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>0.408</v>
+        <v>0.403</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>0.261</v>
+        <v>0.272</v>
       </c>
       <c r="J7" s="1" t="n">
         <v>0.048</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>0.015</v>
+        <v>0.022</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="M7" s="1" t="n">
         <v>0.003</v>
       </c>
       <c r="N7" s="1" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="Q7" s="1" t="n">
-        <v>0.002</v>
-      </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
@@ -794,48 +792,54 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>1</v>
+        <v>0.2974040000000001</v>
       </c>
       <c r="C8" t="n">
         <v>6</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" s="1" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>0.145</v>
+        <v>0.158</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>0.326</v>
+        <v>0.327</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>0.399</v>
+        <v>0.374</v>
       </c>
       <c r="J8" s="1" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.075</v>
       </c>
       <c r="K8" s="1" t="n">
         <v>0.023</v>
       </c>
       <c r="L8" s="1" t="n">
-        <v>0.011</v>
+        <v>0.015</v>
       </c>
       <c r="M8" s="1" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
+        <v>0.002</v>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>0.003</v>
+      </c>
       <c r="O8" s="1" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="P8" s="1" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="Q8" s="1" t="n">
         <v>0.002</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" s="1" t="n">
+        <v>0.003</v>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -847,7 +851,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>1</v>
+        <v>0.296212</v>
       </c>
       <c r="C9" t="n">
         <v>7</v>
@@ -856,49 +860,49 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" s="1" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>0.019</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>0.12</v>
+        <v>0.127</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>0.364</v>
+        <v>0.388</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>0.219</v>
+        <v>0.189</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>0.102</v>
+        <v>0.096</v>
       </c>
       <c r="M9" s="1" t="n">
-        <v>0.062</v>
+        <v>0.061</v>
       </c>
       <c r="N9" s="1" t="n">
-        <v>0.029</v>
+        <v>0.041</v>
       </c>
       <c r="O9" s="1" t="n">
-        <v>0.023</v>
+        <v>0.019</v>
       </c>
       <c r="P9" s="1" t="n">
-        <v>0.017</v>
+        <v>0.022</v>
       </c>
       <c r="Q9" s="1" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="R9" s="1" t="n">
-        <v>0.01</v>
+        <v>0.007</v>
       </c>
       <c r="S9" s="1" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="T9" s="1" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="U9" s="1" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="10">
@@ -908,7 +912,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>1</v>
+        <v>0.2950200000000001</v>
       </c>
       <c r="C10" t="n">
         <v>8</v>
@@ -916,50 +920,48 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" s="1" t="n">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" s="1" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="M10" s="1" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="N10" s="1" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="P10" s="1" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="Q10" s="1" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="R10" s="1" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="S10" s="1" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="T10" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="U10" s="1" t="n">
         <v>0.006</v>
-      </c>
-      <c r="I10" s="1" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="J10" s="1" t="n">
-        <v>0.234</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>0.253</v>
-      </c>
-      <c r="L10" s="1" t="n">
-        <v>0.199</v>
-      </c>
-      <c r="M10" s="1" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="N10" s="1" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="P10" s="1" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="Q10" s="1" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="R10" s="1" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="S10" s="1" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="T10" s="1" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="U10" s="1" t="n">
-        <v>0.004</v>
       </c>
     </row>
     <row r="11">
@@ -969,7 +971,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>1</v>
+        <v>0.2941260000000001</v>
       </c>
       <c r="C11" t="n">
         <v>9</v>
@@ -982,43 +984,43 @@
         <v>0.004</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>0.031</v>
+        <v>0.041</v>
       </c>
       <c r="J11" s="1" t="n">
-        <v>0.191</v>
+        <v>0.168</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>0.266</v>
+        <v>0.252</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>0.18</v>
+        <v>0.217</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>0.094</v>
+        <v>0.107</v>
       </c>
       <c r="N11" s="1" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.063</v>
       </c>
       <c r="O11" s="1" t="n">
-        <v>0.049</v>
+        <v>0.052</v>
       </c>
       <c r="P11" s="1" t="n">
-        <v>0.023</v>
+        <v>0.021</v>
       </c>
       <c r="Q11" s="1" t="n">
-        <v>0.018</v>
+        <v>0.024</v>
       </c>
       <c r="R11" s="1" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="S11" s="1" t="n">
-        <v>0.014</v>
+        <v>0.015</v>
       </c>
       <c r="T11" s="1" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="U11" s="1" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="12">
@@ -1028,7 +1030,7 @@
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>1</v>
+        <v>0.281908</v>
       </c>
       <c r="C12" t="n">
         <v>10</v>
@@ -1039,43 +1041,43 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="J12" s="1" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="L12" s="1" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="M12" s="1" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="N12" s="1" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="P12" s="1" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q12" s="1" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="R12" s="1" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="S12" s="1" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="T12" s="1" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="U12" s="1" t="n">
         <v>0.022</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>0.158</v>
-      </c>
-      <c r="M12" s="1" t="n">
-        <v>0.152</v>
-      </c>
-      <c r="N12" s="1" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="O12" s="1" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="P12" s="1" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="Q12" s="1" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="R12" s="1" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="S12" s="1" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="T12" s="1" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="U12" s="1" t="n">
-        <v>0.03</v>
       </c>
     </row>
     <row r="13">
@@ -1085,7 +1087,7 @@
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>1</v>
+        <v>0.2813120000000001</v>
       </c>
       <c r="C13" t="n">
         <v>11</v>
@@ -1096,53 +1098,53 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="J13" s="1" t="n">
-        <v>0.022</v>
+        <v>0.019</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>0.045</v>
+        <v>0.048</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>0.104</v>
+        <v>0.111</v>
       </c>
       <c r="M13" s="1" t="n">
-        <v>0.164</v>
+        <v>0.149</v>
       </c>
       <c r="N13" s="1" t="n">
-        <v>0.125</v>
+        <v>0.134</v>
       </c>
       <c r="O13" s="1" t="n">
-        <v>0.118</v>
+        <v>0.114</v>
       </c>
       <c r="P13" s="1" t="n">
-        <v>0.104</v>
+        <v>0.105</v>
       </c>
       <c r="Q13" s="1" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.079</v>
       </c>
       <c r="R13" s="1" t="n">
-        <v>0.055</v>
+        <v>0.063</v>
       </c>
       <c r="S13" s="1" t="n">
-        <v>0.04</v>
+        <v>0.049</v>
       </c>
       <c r="T13" s="1" t="n">
-        <v>0.041</v>
+        <v>0.042</v>
       </c>
       <c r="U13" s="1" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Yanchik_250</t>
+          <t>Пиковая Дама</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.9790000000000002</v>
+        <v>0.268796</v>
       </c>
       <c r="C14" t="n">
         <v>12</v>
@@ -1154,50 +1156,50 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" s="1" t="n">
-        <v>0.011</v>
+        <v>0.005</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>0.023</v>
+        <v>0.022</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>0.056</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="M14" s="1" t="n">
-        <v>0.114</v>
+        <v>0.124</v>
       </c>
       <c r="N14" s="1" t="n">
-        <v>0.111</v>
+        <v>0.126</v>
       </c>
       <c r="O14" s="1" t="n">
-        <v>0.115</v>
+        <v>0.122</v>
       </c>
       <c r="P14" s="1" t="n">
-        <v>0.11</v>
+        <v>0.104</v>
       </c>
       <c r="Q14" s="1" t="n">
-        <v>0.107</v>
+        <v>0.091</v>
       </c>
       <c r="R14" s="1" t="n">
-        <v>0.078</v>
+        <v>0.091</v>
       </c>
       <c r="S14" s="1" t="n">
-        <v>0.075</v>
+        <v>0.055</v>
       </c>
       <c r="T14" s="1" t="n">
-        <v>0.049</v>
+        <v>0.051</v>
       </c>
       <c r="U14" s="1" t="n">
-        <v>0.041</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Пиковая Дама</t>
+          <t>Yanchik_250</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.2684980000000001</v>
       </c>
       <c r="C15" t="n">
         <v>13</v>
@@ -1209,50 +1211,50 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" s="1" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="K15" s="1" t="n">
-        <v>0.021</v>
+        <v>0.031</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>0.079</v>
+        <v>0.078</v>
       </c>
       <c r="M15" s="1" t="n">
         <v>0.117</v>
       </c>
       <c r="N15" s="1" t="n">
-        <v>0.141</v>
+        <v>0.125</v>
       </c>
       <c r="O15" s="1" t="n">
-        <v>0.113</v>
+        <v>0.103</v>
       </c>
       <c r="P15" s="1" t="n">
-        <v>0.115</v>
+        <v>0.112</v>
       </c>
       <c r="Q15" s="1" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.083</v>
       </c>
       <c r="R15" s="1" t="n">
-        <v>0.079</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="S15" s="1" t="n">
-        <v>0.048</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="T15" s="1" t="n">
-        <v>0.045</v>
+        <v>0.062</v>
       </c>
       <c r="U15" s="1" t="n">
-        <v>0.031</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cheremsha</t>
+          <t>Laches1</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.9218000000000002</v>
+        <v>0.2488300000000001</v>
       </c>
       <c r="C16" t="n">
         <v>14</v>
@@ -1262,52 +1264,54 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="J16" s="1" t="n">
         <v>0.002</v>
       </c>
       <c r="K16" s="1" t="n">
-        <v>0.017</v>
+        <v>0.015</v>
       </c>
       <c r="L16" s="1" t="n">
-        <v>0.031</v>
+        <v>0.039</v>
       </c>
       <c r="M16" s="1" t="n">
-        <v>0.057</v>
+        <v>0.06</v>
       </c>
       <c r="N16" s="1" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.108</v>
       </c>
       <c r="O16" s="1" t="n">
-        <v>0.103</v>
+        <v>0.113</v>
       </c>
       <c r="P16" s="1" t="n">
-        <v>0.101</v>
+        <v>0.107</v>
       </c>
       <c r="Q16" s="1" t="n">
-        <v>0.113</v>
+        <v>0.116</v>
       </c>
       <c r="R16" s="1" t="n">
-        <v>0.107</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="S16" s="1" t="n">
-        <v>0.095</v>
+        <v>0.068</v>
       </c>
       <c r="T16" s="1" t="n">
-        <v>0.079</v>
+        <v>0.064</v>
       </c>
       <c r="U16" s="1" t="n">
-        <v>0.046</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Laches1</t>
+          <t>cheremsha</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.9075000000000002</v>
+        <v>0.243466</v>
       </c>
       <c r="C17" t="n">
         <v>15</v>
@@ -1319,40 +1323,40 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" s="1" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="K17" s="1" t="n">
-        <v>0.013</v>
+        <v>0.008</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>0.033</v>
+        <v>0.024</v>
       </c>
       <c r="M17" s="1" t="n">
-        <v>0.062</v>
+        <v>0.059</v>
       </c>
       <c r="N17" s="1" t="n">
-        <v>0.097</v>
+        <v>0.078</v>
       </c>
       <c r="O17" s="1" t="n">
-        <v>0.098</v>
+        <v>0.094</v>
       </c>
       <c r="P17" s="1" t="n">
-        <v>0.114</v>
+        <v>0.105</v>
       </c>
       <c r="Q17" s="1" t="n">
-        <v>0.104</v>
+        <v>0.11</v>
       </c>
       <c r="R17" s="1" t="n">
-        <v>0.098</v>
+        <v>0.112</v>
       </c>
       <c r="S17" s="1" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.093</v>
       </c>
       <c r="T17" s="1" t="n">
-        <v>0.062</v>
+        <v>0.075</v>
       </c>
       <c r="U17" s="1" t="n">
-        <v>0.056</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="18">
@@ -1362,7 +1366,7 @@
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.8392999999999999</v>
+        <v>0.230056</v>
       </c>
       <c r="C18" t="n">
         <v>16</v>
@@ -1374,40 +1378,40 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" s="1" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="K18" s="1" t="n">
         <v>0.003</v>
       </c>
-      <c r="K18" s="1" t="n">
-        <v>0.001</v>
-      </c>
       <c r="L18" s="1" t="n">
-        <v>0.02</v>
+        <v>0.016</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>0.051</v>
+        <v>0.034</v>
       </c>
       <c r="N18" s="1" t="n">
-        <v>0.048</v>
+        <v>0.061</v>
       </c>
       <c r="O18" s="1" t="n">
-        <v>0.106</v>
+        <v>0.083</v>
       </c>
       <c r="P18" s="1" t="n">
-        <v>0.113</v>
+        <v>0.104</v>
       </c>
       <c r="Q18" s="1" t="n">
-        <v>0.097</v>
+        <v>0.105</v>
       </c>
       <c r="R18" s="1" t="n">
-        <v>0.097</v>
+        <v>0.112</v>
       </c>
       <c r="S18" s="1" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.099</v>
       </c>
       <c r="T18" s="1" t="n">
-        <v>0.075</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="U18" s="1" t="n">
-        <v>0.064</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="19">
@@ -1417,7 +1421,7 @@
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.7964</v>
+        <v>0.2190300000000001</v>
       </c>
       <c r="C19" t="n">
         <v>17</v>
@@ -1428,39 +1432,41 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="K19" s="1" t="n">
-        <v>0.008</v>
+        <v>0.005</v>
       </c>
       <c r="L19" s="1" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="M19" s="1" t="n">
-        <v>0.031</v>
+        <v>0.041</v>
       </c>
       <c r="N19" s="1" t="n">
-        <v>0.054</v>
+        <v>0.041</v>
       </c>
       <c r="O19" s="1" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="P19" s="1" t="n">
-        <v>0.077</v>
+        <v>0.098</v>
       </c>
       <c r="Q19" s="1" t="n">
-        <v>0.109</v>
+        <v>0.105</v>
       </c>
       <c r="R19" s="1" t="n">
-        <v>0.096</v>
+        <v>0.101</v>
       </c>
       <c r="S19" s="1" t="n">
-        <v>0.095</v>
+        <v>0.107</v>
       </c>
       <c r="T19" s="1" t="n">
-        <v>0.098</v>
+        <v>0.075</v>
       </c>
       <c r="U19" s="1" t="n">
-        <v>0.068</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1470,7 +1476,7 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.4455000000000001</v>
+        <v>0.12069</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>18</v>
@@ -1483,43 +1489,45 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="3" t="n">
+        <v>0.001</v>
+      </c>
       <c r="M20" s="3" t="n">
-        <v>0.002</v>
+        <v>0.006</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.012</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.016</v>
+        <v>0.02</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.037</v>
+        <v>0.027</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.035</v>
+        <v>0.044</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.056</v>
+        <v>0.054</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0.076</v>
+        <v>0.058</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.075</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.096</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>nesmotri_v_shelll1</t>
+          <t>ksuhony</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.3927</v>
+        <v>0.105194</v>
       </c>
       <c r="C21" t="n">
         <v>19</v>
@@ -1532,45 +1540,43 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" s="1" t="n">
         <v>0.003</v>
       </c>
       <c r="N21" s="1" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="O21" s="1" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.013</v>
       </c>
       <c r="P21" s="1" t="n">
-        <v>0.023</v>
+        <v>0.02</v>
       </c>
       <c r="Q21" s="1" t="n">
-        <v>0.028</v>
+        <v>0.027</v>
       </c>
       <c r="R21" s="1" t="n">
-        <v>0.057</v>
+        <v>0.048</v>
       </c>
       <c r="S21" s="1" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="T21" s="1" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.083</v>
       </c>
       <c r="U21" s="1" t="n">
-        <v>0.081</v>
+        <v>0.095</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ksuhony</t>
+          <t>nesmotri_v_shelll1</t>
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.3872</v>
+        <v>0.09476400000000003</v>
       </c>
       <c r="C22" t="n">
         <v>20</v>
@@ -1584,12 +1590,14 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" s="1" t="n">
+        <v>0.002</v>
+      </c>
       <c r="N22" s="1" t="n">
-        <v>0.002</v>
+        <v>0.006</v>
       </c>
       <c r="O22" s="1" t="n">
-        <v>0.006</v>
+        <v>0.012</v>
       </c>
       <c r="P22" s="1" t="n">
         <v>0.016</v>
@@ -1598,16 +1606,16 @@
         <v>0.033</v>
       </c>
       <c r="R22" s="1" t="n">
-        <v>0.057</v>
+        <v>0.04</v>
       </c>
       <c r="S22" s="1" t="n">
-        <v>0.067</v>
+        <v>0.061</v>
       </c>
       <c r="T22" s="1" t="n">
-        <v>0.076</v>
+        <v>0.061</v>
       </c>
       <c r="U22" s="1" t="n">
-        <v>0.095</v>
+        <v>0.08699999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1617,7 +1625,7 @@
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.3069000000000001</v>
+        <v>0.08612200000000002</v>
       </c>
       <c r="C23" t="n">
         <v>21</v>
@@ -1631,30 +1639,32 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" s="1" t="n">
+        <v>0.002</v>
+      </c>
       <c r="N23" s="1" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="O23" s="1" t="n">
-        <v>0.008</v>
+        <v>0.002</v>
       </c>
       <c r="P23" s="1" t="n">
-        <v>0.016</v>
+        <v>0.02</v>
       </c>
       <c r="Q23" s="1" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="R23" s="1" t="n">
-        <v>0.028</v>
+        <v>0.034</v>
       </c>
       <c r="S23" s="1" t="n">
-        <v>0.055</v>
+        <v>0.062</v>
       </c>
       <c r="T23" s="1" t="n">
-        <v>0.066</v>
+        <v>0.061</v>
       </c>
       <c r="U23" s="1" t="n">
-        <v>0.077</v>
+        <v>0.076</v>
       </c>
     </row>
     <row r="24">
@@ -1664,7 +1674,7 @@
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>0.2816</v>
+        <v>0.073606</v>
       </c>
       <c r="C24" t="n">
         <v>22</v>
@@ -1676,29 +1686,33 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" s="1" t="n">
+        <v>0.002</v>
+      </c>
       <c r="N24" s="1" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="O24" s="1" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
       <c r="P24" s="1" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="Q24" s="1" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="R24" s="1" t="n">
-        <v>0.051</v>
+        <v>0.032</v>
       </c>
       <c r="S24" s="1" t="n">
-        <v>0.041</v>
+        <v>0.047</v>
       </c>
       <c r="T24" s="1" t="n">
-        <v>0.068</v>
+        <v>0.065</v>
       </c>
       <c r="U24" s="1" t="n">
         <v>0.063</v>
@@ -1707,11 +1721,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gvrdkn</t>
+          <t>sfv</t>
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>0.2002</v>
+        <v>0.055726</v>
       </c>
       <c r="C25" t="n">
         <v>23</v>
@@ -1728,35 +1742,35 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" s="1" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="P25" s="1" t="n">
         <v>0.005</v>
       </c>
       <c r="Q25" s="1" t="n">
-        <v>0.016</v>
+        <v>0.006</v>
       </c>
       <c r="R25" s="1" t="n">
-        <v>0.021</v>
+        <v>0.028</v>
       </c>
       <c r="S25" s="1" t="n">
-        <v>0.026</v>
+        <v>0.029</v>
       </c>
       <c r="T25" s="1" t="n">
-        <v>0.046</v>
+        <v>0.054</v>
       </c>
       <c r="U25" s="1" t="n">
-        <v>0.067</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Julia_2499</t>
+          <t>gvrdkn</t>
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>0.1969</v>
+        <v>0.049766</v>
       </c>
       <c r="C26" t="n">
         <v>24</v>
@@ -1769,41 +1783,45 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+      <c r="L26" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M26" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="N26" s="1" t="n">
         <v>0.001</v>
       </c>
       <c r="O26" s="1" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="P26" s="1" t="n">
         <v>0.005</v>
       </c>
-      <c r="P26" s="1" t="n">
-        <v>0.01</v>
-      </c>
       <c r="Q26" s="1" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="R26" s="1" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="S26" s="1" t="n">
-        <v>0.034</v>
+        <v>0.036</v>
       </c>
       <c r="T26" s="1" t="n">
-        <v>0.047</v>
+        <v>0.043</v>
       </c>
       <c r="U26" s="1" t="n">
-        <v>0.056</v>
+        <v>0.046</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sfv</t>
+          <t>Julia_2499</t>
         </is>
       </c>
       <c r="B27" s="1" t="n">
-        <v>0.1881</v>
+        <v>0.04946800000000001</v>
       </c>
       <c r="C27" t="n">
         <v>25</v>
@@ -1817,30 +1835,30 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="N27" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="O27" s="1" t="n">
-        <v>0.003</v>
-      </c>
+        <v>0.002</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" s="1" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="Q27" s="1" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="R27" s="1" t="n">
-        <v>0.023</v>
+        <v>0.02</v>
       </c>
       <c r="S27" s="1" t="n">
-        <v>0.023</v>
+        <v>0.031</v>
       </c>
       <c r="T27" s="1" t="n">
-        <v>0.05</v>
+        <v>0.039</v>
       </c>
       <c r="U27" s="1" t="n">
-        <v>0.056</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="28">
@@ -1850,7 +1868,7 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>0.05280000000000001</v>
+        <v>0.012814</v>
       </c>
       <c r="C28" t="n">
         <v>26</v>
@@ -1866,34 +1884,30 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" s="1" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="P28" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" s="1" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="S28" s="1" t="n">
         <v>0.005</v>
       </c>
       <c r="T28" s="1" t="n">
-        <v>0.012</v>
+        <v>0.016</v>
       </c>
       <c r="U28" s="1" t="n">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1С</t>
+          <t>Davit</t>
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0005960000000000001</v>
       </c>
       <c r="C29" t="n">
         <v>27</v>
@@ -1912,27 +1926,23 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" s="1" t="n">
-        <v>0.001</v>
-      </c>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="T29" s="1" t="n">
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" s="1" t="n">
         <v>0.001</v>
-      </c>
-      <c r="U29" s="1" t="n">
-        <v>0.005</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Настя дай стек</t>
+          <t>БОЛЬШОЙ МИХА</t>
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>0.0011</v>
+        <v>0.000298</v>
       </c>
       <c r="C30" t="n">
         <v>28</v>
@@ -1952,20 +1962,20 @@
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
-      <c r="S30" s="1" t="n">
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" s="1" t="n">
         <v>0.001</v>
       </c>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Davit</t>
+          <t>1С</t>
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>0.0011</v>
+        <v>0.000298</v>
       </c>
       <c r="C31" t="n">
         <v>29</v>
@@ -1985,19 +1995,21 @@
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" s="1" t="n">
+      <c r="S31" s="1" t="n">
         <v>0.001</v>
       </c>
+      <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>БОЛЬШОЙ МИХА</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>bogdanov</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>0.000298</v>
+      </c>
       <c r="C32" t="n">
         <v>30</v>
       </c>
@@ -2017,13 +2029,15 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
+      <c r="T32" s="1" t="n">
+        <v>0.001</v>
+      </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Davydovpussy</t>
+          <t>Suruchik</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -2052,7 +2066,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alina_97</t>
+          <t>.</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -2081,7 +2095,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>springbulk</t>
+          <t>Son_Ton</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -2110,7 +2124,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Son_Ton</t>
+          <t>Настя дай стек</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -2139,7 +2153,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cordell</t>
+          <t>Yars</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -2168,7 +2182,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Suruchik</t>
+          <t>Аннэтт</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -2197,7 +2211,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Retbin</t>
+          <t>Alina_97</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -2226,7 +2240,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Yars</t>
+          <t>Cordell</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -2255,7 +2269,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Аннэтт</t>
+          <t>Davydovpussy</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -2284,7 +2298,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DARI</t>
+          <t>Qrexi</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -2313,7 +2327,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>mflameee</t>
+          <t>Адольф</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -2342,7 +2356,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>bogdanov</t>
+          <t>DARI</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2371,7 +2385,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ryumon_Hozukimaruu</t>
+          <t>Никита</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -2400,7 +2414,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Никита</t>
+          <t>Retbin</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -2429,7 +2443,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mar_u_shka</t>
+          <t>Gur4an</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -2458,7 +2472,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rik_dds</t>
+          <t>Ryumon_Hozukimaruu</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -2487,7 +2501,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>mrCelviano</t>
+          <t>springbulk</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -2516,7 +2530,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Serg</t>
+          <t>mrCelviano</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2545,7 +2559,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>Rik_dds</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2574,7 +2588,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>repe_kate</t>
+          <t>He3hAy</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>

</xml_diff>